<commit_message>
ops: add 40 secondary routines to PLAYBOOK_COCKPIT (199 total)
New categories added:
- Linear & Ticket Management (5): TMS v2.0, state flow, ownership
- Escalação & Comunicação (6): escalation by issue type, Slack map, SLA
- Aprovações & Sign-off (4): gate approvers, SOW, feature sign-off
- Decisões & Documentação (4): decision log, context recovery
- Monitoramento & Cadência (5): weekly blockers, bi-weekly cortex
- Regras Operacionais Críticas (8): IES=all, wait 30-45s, no secrets
- Gaps Secundários (8): SLA, TSA↔Eng boundary, dataset criteria

Totals: 199 routines | 84 SIM | 113 NÃO | 142 INCLUIR | 25 EXCLUIR | 32 PENDENTE | 16 GAPs

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLAYBOOK_COCKPIT.xlsx
+++ b/PLAYBOOK_COCKPIT.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,14 @@
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -140,6 +146,12 @@
         <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -167,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,6 +230,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -591,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10016,129 +10031,2561 @@
         </is>
       </c>
     </row>
-    <row r="180" ht="24" customHeight="1">
-      <c r="A180" s="18" t="inlineStr">
+    <row r="179" ht="24" customHeight="1">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>LINEAR &amp; TICKET MANAGEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="B180" s="8" t="inlineStr">
+        <is>
+          <t>Linear/Tickets</t>
+        </is>
+      </c>
+      <c r="C180" s="8" t="inlineStr">
+        <is>
+          <t>Quando criar ticket Linear</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>Novo task, bug, blocker, feature request → sempre ticket</t>
+        </is>
+      </c>
+      <c r="E180" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F180" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md</t>
+        </is>
+      </c>
+      <c r="G180" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J180" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K180" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L180" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Regra fundamental não documentada no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="3" t="n">
+        <v>161</v>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>Linear/Tickets</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>TMS v2.0 (10-point ticket audit)</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>Title, AC, assignee, milestone, deps, estimate, blockers, SOW trace, no dupes, state</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="F181" s="4" t="inlineStr">
+        <is>
+          <t>FULL_IMPLEMENTATION_PROCESS.md</t>
+        </is>
+      </c>
+      <c r="G181" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J181" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K181" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L181" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Checklist de qualidade de ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="8" t="n">
+        <v>162</v>
+      </c>
+      <c r="B182" s="8" t="inlineStr">
+        <is>
+          <t>Linear/Tickets</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="inlineStr">
+        <is>
+          <t>State Flow padrão</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>Clear → Backlog → Refinement → Engineering → Done</t>
+        </is>
+      </c>
+      <c r="E182" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F182" s="9" t="inlineStr">
+        <is>
+          <t>FULL_IMPLEMENTATION_PROCESS.md</t>
+        </is>
+      </c>
+      <c r="G182" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J182" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K182" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L182" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: TSA owns até Backlog, Eng owns de Refinement em diante</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="3" t="n">
+        <v>163</v>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>Linear/Tickets</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>Ownership boundary (TSA vs Eng)</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>TSA owns ticket até Backlog; Engineering owns de Refinement forward</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="inlineStr">
+        <is>
+          <t>FULL_IMPLEMENTATION_PROCESS.md</t>
+        </is>
+      </c>
+      <c r="G183" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J183" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K183" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L183" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Quem é dono de quê em cada fase</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="B184" s="8" t="inlineStr">
+        <is>
+          <t>Linear/Tickets</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t>Batch ticket update scripts</t>
+        </is>
+      </c>
+      <c r="D184" s="9" t="inlineStr">
+        <is>
+          <t>linear_update.py, linear_update_all.py, get_full_ticket_table.py</t>
+        </is>
+      </c>
+      <c r="E184" s="8" t="inlineStr">
+        <is>
+          <t>Reusável</t>
+        </is>
+      </c>
+      <c r="F184" s="9" t="inlineStr">
+        <is>
+          <t>scripts/ingestion/linear_*.py</t>
+        </is>
+      </c>
+      <c r="G184" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J184" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K184" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L184" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Scripts de automação Linear</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="24" customHeight="1">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>ESCALAÇÃO &amp; COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>Escalation Path por tipo de issue</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>Feature→Katherine; Eng→Lucas/Augusto; Data→Alexandra; Decisions→Katherine/Christina</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/07_CONTACTS_AND_STAKEHOLDERS.md</t>
+        </is>
+      </c>
+      <c r="G186" s="18" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>Cap 12</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>Simplificado</t>
+        </is>
+      </c>
+      <c r="J186" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K186" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Playbook tem 4 níveis genéricos mas NÃO detalha por tipo de issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="8" t="n">
+        <v>166</v>
+      </c>
+      <c r="B187" s="8" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t>Regra de 1 semana (blocker escalation)</t>
+        </is>
+      </c>
+      <c r="D187" s="9" t="inlineStr">
+        <is>
+          <t>Se blocker &gt;1 semana sem progresso → escalar para Katherine</t>
+        </is>
+      </c>
+      <c r="E187" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F187" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/08_RISK_MATRIX_AND_BLOCKERS.md</t>
+        </is>
+      </c>
+      <c r="G187" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J187" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K187" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L187" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Regra temporal de escalação NÃO no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="30" customHeight="1">
+      <c r="A188" s="3" t="n">
+        <v>167</v>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Slack Channels por contexto</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>#testbox-intuit-mm-external, #intuit-internal, #testbox-eng, #tsa-internal, #wfs-internal</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>Referência</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/07_CONTACTS_AND_STAKEHOLDERS.md</t>
+        </is>
+      </c>
+      <c r="G188" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J188" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K188" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L188" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Onde postar cada tipo de mensagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="30" customHeight="1">
+      <c r="A189" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="B189" s="8" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C189" s="8" t="inlineStr">
+        <is>
+          <t>Communication Map (quem contactar para quê)</t>
+        </is>
+      </c>
+      <c r="D189" s="9" t="inlineStr">
+        <is>
+          <t>Feature→KB→Linear→Katherine; Eng→Lucas→Augusto; Data→Alexandra→TSA Lead</t>
+        </is>
+      </c>
+      <c r="E189" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F189" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/07_CONTACTS_AND_STAKEHOLDERS.md</t>
+        </is>
+      </c>
+      <c r="G189" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H189" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I189" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J189" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K189" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L189" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Mapa completo de comunicação por tipo de problema</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="30" customHeight="1">
+      <c r="A190" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>IES Release Communication Flow</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>Siji George → 'Write it Straight' doc → UAT doc → Feature Activation</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/07_CONTACTS_AND_STAKEHOLDERS.md</t>
+        </is>
+      </c>
+      <c r="G190" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H190" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I190" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J190" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K190" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L190" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Fluxo específico Intuit para ativação de features</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="B191" s="8" t="inlineStr">
+        <is>
+          <t>Escalação</t>
+        </is>
+      </c>
+      <c r="C191" s="8" t="inlineStr">
+        <is>
+          <t>SLA de resposta por prioridade</t>
+        </is>
+      </c>
+      <c r="D191" s="9" t="inlineStr">
+        <is>
+          <t>P0: 4h, P1: 24h, P2: 1 semana — não documentado formalmente</t>
+        </is>
+      </c>
+      <c r="E191" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F191" s="9" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G191" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H191" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I191" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J191" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K191" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L191" s="9" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: SLA informal mas não formalizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="24" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>APROVAÇÕES &amp; SIGN-OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="30" customHeight="1">
+      <c r="A193" s="3" t="n">
+        <v>171</v>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>Aprovações</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>Gate sign-off (quem aprova cada gate)</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>Gate 1: TSA, Gate 2: Backend Eng, Gate 3: Claude, Feature: Eng Lead/PO</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t>INGESTION_3_GATES.md + FULL_IMPLEMENTATION_PROCESS.md</t>
+        </is>
+      </c>
+      <c r="G193" s="18" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="H193" s="3" t="inlineStr">
+        <is>
+          <t>Cap 5</t>
+        </is>
+      </c>
+      <c r="I193" s="3" t="inlineStr">
+        <is>
+          <t>Implícito</t>
+        </is>
+      </c>
+      <c r="J193" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K193" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L193" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Playbook descreve gates mas NÃO explicita quem aprova cada um</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="30" customHeight="1">
+      <c r="A194" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>Aprovações</t>
+        </is>
+      </c>
+      <c r="C194" s="8" t="inlineStr">
+        <is>
+          <t>SOW approval workflow</t>
+        </is>
+      </c>
+      <c r="D194" s="9" t="inlineStr">
+        <is>
+          <t>Commercial propõe → Katherine aprova → TSA executa</t>
+        </is>
+      </c>
+      <c r="E194" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F194" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/03_SOW_AND_SCOPE.md</t>
+        </is>
+      </c>
+      <c r="G194" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H194" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I194" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J194" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K194" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L194" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Quem aprova o escopo</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="30" customHeight="1">
+      <c r="A195" s="3" t="n">
+        <v>173</v>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Aprovações</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Environment decision approval</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>Christina Duarte (WFS), Katherine (timeline), Sam (engineering invest.)</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/10_DECISIONS_LOG.md</t>
+        </is>
+      </c>
+      <c r="G195" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I195" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J195" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K195" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L195" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Quem decide sobre ambientes e investimentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="A196" s="8" t="n">
+        <v>174</v>
+      </c>
+      <c r="B196" s="8" t="inlineStr">
+        <is>
+          <t>Aprovações</t>
+        </is>
+      </c>
+      <c r="C196" s="8" t="inlineStr">
+        <is>
+          <t>Feature validation sign-off criteria</t>
+        </is>
+      </c>
+      <c r="D196" s="9" t="inlineStr">
+        <is>
+          <t>Data quality strong, all variants captured, envs compared → Eng Lead aprova</t>
+        </is>
+      </c>
+      <c r="E196" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F196" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md</t>
+        </is>
+      </c>
+      <c r="G196" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H196" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I196" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J196" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K196" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L196" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Critérios de aceite para validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="24" customHeight="1">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>DECISÕES &amp; DOCUMENTAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="30" customHeight="1">
+      <c r="A198" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>Decisões</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>Decision Log protocol</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>Toda decisão material → registrar ID, date, who, why, impact</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F198" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/10_DECISIONS_LOG.md</t>
+        </is>
+      </c>
+      <c r="G198" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H198" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J198" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K198" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L198" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Obrigatório mas NÃO mencionado no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="30" customHeight="1">
+      <c r="A199" s="8" t="n">
+        <v>176</v>
+      </c>
+      <c r="B199" s="8" t="inlineStr">
+        <is>
+          <t>Decisões</t>
+        </is>
+      </c>
+      <c r="C199" s="8" t="inlineStr">
+        <is>
+          <t>Pending Decisions tracking</t>
+        </is>
+      </c>
+      <c r="D199" s="9" t="inlineStr">
+        <is>
+          <t>P-001 WFS env, P-002 Manufacturing, P-003 Demo Health — awaiting owners</t>
+        </is>
+      </c>
+      <c r="E199" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F199" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/10_DECISIONS_LOG.md</t>
+        </is>
+      </c>
+      <c r="G199" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H199" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I199" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J199" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K199" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L199" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Específico vs genérico no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="30" customHeight="1">
+      <c r="A200" s="3" t="n">
+        <v>177</v>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>Decisões</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>Session finalization (/consolidar)</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>memory.md + session file + git commit + push — OBRIGATÓRIO</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F200" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md</t>
+        </is>
+      </c>
+      <c r="G200" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="inlineStr">
+        <is>
+          <t>Cap 12</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>Mencionado</t>
+        </is>
+      </c>
+      <c r="J200" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K200" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L200" s="4" t="inlineStr"/>
+    </row>
+    <row r="201" ht="30" customHeight="1">
+      <c r="A201" s="8" t="n">
+        <v>178</v>
+      </c>
+      <c r="B201" s="8" t="inlineStr">
+        <is>
+          <t>Decisões</t>
+        </is>
+      </c>
+      <c r="C201" s="8" t="inlineStr">
+        <is>
+          <t>Context Recovery protocol</t>
+        </is>
+      </c>
+      <c r="D201" s="9" t="inlineStr">
+        <is>
+          <t>Startup: OUTPUT_A → memory.md → CLAUDE.md → sessions/</t>
+        </is>
+      </c>
+      <c r="E201" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F201" s="9" t="inlineStr">
+        <is>
+          <t>knowledge-base/CONTEXT_RECOVERY.md</t>
+        </is>
+      </c>
+      <c r="G201" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H201" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I201" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J201" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K201" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L201" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Como recuperar contexto entre sessões</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="24" customHeight="1">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAMENTO &amp; CADÊNCIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="30" customHeight="1">
+      <c r="A203" s="3" t="n">
+        <v>179</v>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>Monitoramento</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Weekly Blocker Review</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>Linear filter 'Blocked' → check status → update memory → escalate se &gt;1sem</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md (Runbook 11)</t>
+        </is>
+      </c>
+      <c r="G203" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J203" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K203" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L203" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Rotina semanal obrigatória não no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="30" customHeight="1">
+      <c r="A204" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="B204" s="8" t="inlineStr">
+        <is>
+          <t>Monitoramento</t>
+        </is>
+      </c>
+      <c r="C204" s="8" t="inlineStr">
+        <is>
+          <t>Weekly Monitoring Checklist</t>
+        </is>
+      </c>
+      <c r="D204" s="9" t="inlineStr">
+        <is>
+          <t>Ingestion CSVs, WFS decision, Linear progress, new blockers</t>
+        </is>
+      </c>
+      <c r="E204" s="8" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="F204" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/08_RISK_MATRIX_AND_BLOCKERS.md</t>
+        </is>
+      </c>
+      <c r="G204" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H204" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I204" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J204" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K204" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L204" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: 4 items semanais obrigatórios</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="30" customHeight="1">
+      <c r="A205" s="3" t="n">
+        <v>181</v>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Monitoramento</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Bi-weekly Strategic Cortex update</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr">
+        <is>
+          <t>TSA_CORTEX collect --all → 5 outputs → publish</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md (Runbook 10)</t>
+        </is>
+      </c>
+      <c r="G205" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J205" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K205" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L205" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Atualização quinzenal de inteligência</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="30" customHeight="1">
+      <c r="A206" s="8" t="n">
+        <v>182</v>
+      </c>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Monitoramento</t>
+        </is>
+      </c>
+      <c r="C206" s="8" t="inlineStr">
+        <is>
+          <t>Pre-Release verification cadence</t>
+        </is>
+      </c>
+      <c r="D206" s="9" t="inlineStr">
+        <is>
+          <t>All features, foundation data, feature flags, validation framework</t>
+        </is>
+      </c>
+      <c r="E206" s="8" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="F206" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/08_RISK_MATRIX_AND_BLOCKERS.md</t>
+        </is>
+      </c>
+      <c r="G206" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H206" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I206" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J206" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K206" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L206" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: O que verificar antes de cada release</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="30" customHeight="1">
+      <c r="A207" s="3" t="n">
+        <v>183</v>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>Monitoramento</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Activity Plan 24h monitoring</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>Retool → check next_execution_at → se &gt;24h → alert</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F207" s="4" t="inlineStr">
+        <is>
+          <t>Cap 11 (inline) + DGO-652</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>Cap 11</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>Detalhado</t>
+        </is>
+      </c>
+      <c r="J207" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K207" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L207" s="4" t="inlineStr"/>
+    </row>
+    <row r="208" ht="24" customHeight="1">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>REGRAS OPERACIONAIS CRÍTICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="30" customHeight="1">
+      <c r="A209" s="8" t="n">
+        <v>184</v>
+      </c>
+      <c r="B209" s="8" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C209" s="8" t="inlineStr">
+        <is>
+          <t>IES = ALL features (não subset)</t>
+        </is>
+      </c>
+      <c r="D209" s="9" t="inlineStr">
+        <is>
+          <t>IES validation deve cobrir TODAS features, erro histórico de pular</t>
+        </is>
+      </c>
+      <c r="E209" s="8" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F209" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md</t>
+        </is>
+      </c>
+      <c r="G209" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H209" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I209" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J209" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K209" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L209" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Regra aprendida com erro — obrigatória</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="30" customHeight="1">
+      <c r="A210" s="3" t="n">
+        <v>185</v>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Wait 30-45s (não 10s) no QBO SPA</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>QBO SPA é lento, 10s = screenshot de loading state</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F210" s="4" t="inlineStr">
+        <is>
+          <t>PROMPT_CLAUDE_QBO_MASTER.md</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>Cap 7, 9</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>Mencionado</t>
+        </is>
+      </c>
+      <c r="J210" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K210" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L210" s="4" t="inlineStr"/>
+    </row>
+    <row r="211" ht="30" customHeight="1">
+      <c r="A211" s="8" t="n">
+        <v>186</v>
+      </c>
+      <c r="B211" s="8" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C211" s="8" t="inlineStr">
+        <is>
+          <t>Screenshot &gt;100KB = válido, ~140KB = 404</t>
+        </is>
+      </c>
+      <c r="D211" s="9" t="inlineStr">
+        <is>
+          <t>Validação de tamanho de arquivo para detectar erros</t>
+        </is>
+      </c>
+      <c r="E211" s="8" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F211" s="9" t="inlineStr">
+        <is>
+          <t>EVIDENCE_COLLECTION_PLAYBOOK.md</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H211" s="8" t="inlineStr">
+        <is>
+          <t>Cap 9</t>
+        </is>
+      </c>
+      <c r="I211" s="8" t="inlineStr">
+        <is>
+          <t>Detalhado</t>
+        </is>
+      </c>
+      <c r="J211" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K211" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L211" s="9" t="inlineStr"/>
+    </row>
+    <row r="212" ht="30" customHeight="1">
+      <c r="A212" s="3" t="n">
+        <v>187</v>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>NEVER print passwords/TOTP in chat</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>Segurança: credenciais nunca expostas em output</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>PROMPT_CLAUDE_QBO_MASTER.md</t>
+        </is>
+      </c>
+      <c r="G212" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J212" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K212" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L212" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Regra de segurança crítica não no playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="30" customHeight="1">
+      <c r="A213" s="8" t="n">
+        <v>188</v>
+      </c>
+      <c r="B213" s="8" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C213" s="8" t="inlineStr">
+        <is>
+          <t>No advance without gate PASS</t>
+        </is>
+      </c>
+      <c r="D213" s="9" t="inlineStr">
+        <is>
+          <t>Gate anterior DEVE passar antes de avançar para próximo</t>
+        </is>
+      </c>
+      <c r="E213" s="8" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F213" s="9" t="inlineStr">
+        <is>
+          <t>INGESTION_3_GATES.md</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H213" s="8" t="inlineStr">
+        <is>
+          <t>Cap 5</t>
+        </is>
+      </c>
+      <c r="I213" s="8" t="inlineStr">
+        <is>
+          <t>Implícito</t>
+        </is>
+      </c>
+      <c r="J213" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K213" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L213" s="9" t="inlineStr"/>
+    </row>
+    <row r="214" ht="30" customHeight="1">
+      <c r="A214" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Commit learnings after every sweep</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>Sweep sem commit = incompleto, regra do PROMPT_MASTER seção 14.2</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F214" s="4" t="inlineStr">
+        <is>
+          <t>PROMPT_CLAUDE_QBO_MASTER.md</t>
+        </is>
+      </c>
+      <c r="G214" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>Cap 8</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>Detalhado</t>
+        </is>
+      </c>
+      <c r="J214" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K214" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L214" s="4" t="inlineStr"/>
+    </row>
+    <row r="215" ht="30" customHeight="1">
+      <c r="A215" s="8" t="n">
+        <v>190</v>
+      </c>
+      <c r="B215" s="8" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C215" s="8" t="inlineStr">
+        <is>
+          <t>Tentar 3+ rotas antes de marcar N/A</t>
+        </is>
+      </c>
+      <c r="D215" s="9" t="inlineStr">
+        <is>
+          <t>Feature indisponível = tentar URL direta, sidebar, search antes de dar up</t>
+        </is>
+      </c>
+      <c r="E215" s="8" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F215" s="9" t="inlineStr">
+        <is>
+          <t>INTUIT_BOOM_TRANSFER/06_RUNBOOKS.md</t>
+        </is>
+      </c>
+      <c r="G215" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H215" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I215" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J215" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K215" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L215" s="9" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Regra de resiliência na validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="30" customHeight="1">
+      <c r="A216" s="3" t="n">
+        <v>191</v>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Every error = permanent learning</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>Cada erro novo no Retool deve ser documentado permanentemente</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="F216" s="4" t="inlineStr">
+        <is>
+          <t>INGESTION_3_GATES.md</t>
+        </is>
+      </c>
+      <c r="G216" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J216" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K216" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L216" s="4" t="inlineStr">
+        <is>
+          <t>SECUNDÁRIA: Cultura de documentação de erros</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="24" customHeight="1">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>GAPS SECUNDÁRIOS (não documentados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="30" customHeight="1">
+      <c r="A218" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="B218" s="8" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C218" s="8" t="inlineStr">
+        <is>
+          <t>Quando criar novo dataset vs reusar</t>
+        </is>
+      </c>
+      <c r="D218" s="9" t="inlineStr">
+        <is>
+          <t>Critérios para decidir se dataset existente serve ou precisa novo</t>
+        </is>
+      </c>
+      <c r="E218" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F218" s="9" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G218" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H218" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I218" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J218" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K218" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L218" s="9" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Decisão frequente sem critério formal</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="30" customHeight="1">
+      <c r="A219" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>SLA formal por prioridade (P0-P3)</t>
+        </is>
+      </c>
+      <c r="D219" s="4" t="inlineStr">
+        <is>
+          <t>Tempos de resposta esperados por nível de prioridade</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F219" s="4" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G219" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J219" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K219" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L219" s="4" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: SLA informal, precisa formalizar</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="30" customHeight="1">
+      <c r="A220" s="8" t="n">
+        <v>194</v>
+      </c>
+      <c r="B220" s="8" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C220" s="8" t="inlineStr">
+        <is>
+          <t>Handoff TSA↔Engineering (ownership boundary)</t>
+        </is>
+      </c>
+      <c r="D220" s="9" t="inlineStr">
+        <is>
+          <t>Momento exato onde responsabilidade passa de TSA para Eng</t>
+        </is>
+      </c>
+      <c r="E220" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F220" s="9" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G220" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H220" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I220" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J220" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K220" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L220" s="9" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Boundary de ownership não definido</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="30" customHeight="1">
+      <c r="A221" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Quando triggar retrospectiva</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>Critérios: pós-release? pós-sweep &lt;6? pós-incidente?</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F221" s="4" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G221" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J221" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K221" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L221" s="4" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Retro ad-hoc, sem trigger definido</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="30" customHeight="1">
+      <c r="A222" s="8" t="n">
+        <v>196</v>
+      </c>
+      <c r="B222" s="8" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C222" s="8" t="inlineStr">
+        <is>
+          <t>Offboarding / revogar acessos</t>
+        </is>
+      </c>
+      <c r="D222" s="9" t="inlineStr">
+        <is>
+          <t>Quando alguém sai, quais acessos revogar e como</t>
+        </is>
+      </c>
+      <c r="E222" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F222" s="9" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G222" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H222" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I222" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J222" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K222" s="8" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L222" s="9" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Contrário do onboarding</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="30" customHeight="1">
+      <c r="A223" s="3" t="n">
+        <v>197</v>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>Notificação de stakeholders (quando e como)</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr">
+        <is>
+          <t>Quem notificar em cada tipo de evento (fix, blocker, release, demo)</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F223" s="4" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G223" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J223" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K223" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L223" s="4" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Protocolo de notificação por evento</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="30" customHeight="1">
+      <c r="A224" s="8" t="n">
+        <v>198</v>
+      </c>
+      <c r="B224" s="8" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C224" s="8" t="inlineStr">
+        <is>
+          <t>Pair session vs solo (quando pedir help)</t>
+        </is>
+      </c>
+      <c r="D224" s="9" t="inlineStr">
+        <is>
+          <t>Critérios para trabalhar solo vs pedir pair com outro TSA/CE</t>
+        </is>
+      </c>
+      <c r="E224" s="8" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F224" s="9" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G224" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H224" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I224" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J224" s="12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="K224" s="8" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L224" s="9" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Guideline de colaboração</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="30" customHeight="1">
+      <c r="A225" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>GAP Sec.</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Quando atualizar Coda vs Linear vs Drive</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="inlineStr">
+        <is>
+          <t>Qual ferramenta atualizar para cada tipo de informação</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>Protocolo</t>
+        </is>
+      </c>
+      <c r="F225" s="4" t="inlineStr">
+        <is>
+          <t>NÃO EXISTE</t>
+        </is>
+      </c>
+      <c r="G225" s="10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J225" s="6" t="inlineStr">
+        <is>
+          <t>INCLUIR</t>
+        </is>
+      </c>
+      <c r="K225" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L225" s="4" t="inlineStr">
+        <is>
+          <t>GAP SECUNDÁRIA: Mapa de ferramentas por tipo de update</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="24" customHeight="1">
+      <c r="A227" s="19" t="inlineStr">
         <is>
           <t>RESUMO</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="B181" s="19" t="inlineStr">
+    <row r="228">
+      <c r="B228" s="20" t="inlineStr">
         <is>
           <t>Total de rotinas mapeadas</t>
         </is>
       </c>
-      <c r="C181" s="13" t="n">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="B182" s="19" t="inlineStr">
+      <c r="C228" s="13" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="B229" s="20" t="inlineStr">
         <is>
           <t>Já no Playbook (SIM)</t>
         </is>
       </c>
-      <c r="C182" s="13" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="B183" s="19" t="inlineStr">
+      <c r="C229" s="13" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="B230" s="20" t="inlineStr">
         <is>
           <t>Faltando no Playbook (NÃO)</t>
         </is>
       </c>
-      <c r="C183" s="13" t="n">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="B184" s="19" t="inlineStr">
+      <c r="C230" s="13" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="B231" s="20" t="inlineStr">
         <is>
           <t>Decisão: INCLUIR</t>
         </is>
       </c>
-      <c r="C184" s="13" t="n">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="B185" s="19" t="inlineStr">
+      <c r="C231" s="13" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="B232" s="20" t="inlineStr">
         <is>
           <t>Decisão: EXCLUIR</t>
         </is>
       </c>
-      <c r="C185" s="13" t="n">
+      <c r="C232" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="186">
-      <c r="B186" s="19" t="inlineStr">
+    <row r="233">
+      <c r="B233" s="20" t="inlineStr">
         <is>
           <t>Decisão: PENDENTE</t>
         </is>
       </c>
-      <c r="C186" s="13" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="B187" s="19" t="inlineStr">
+      <c r="C233" s="13" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="B234" s="20" t="inlineStr">
         <is>
           <t>Gaps identificados (não existem)</t>
         </is>
       </c>
-      <c r="C187" s="13" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="B188" s="19" t="inlineStr">
+      <c r="C234" s="13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="B235" s="20" t="inlineStr">
         <is>
           <t>Cobertura atual</t>
         </is>
       </c>
-      <c r="C188" s="13" t="inlineStr">
-        <is>
-          <t>78/159 (49%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="B189" s="19" t="inlineStr">
+      <c r="C235" s="13" t="inlineStr">
+        <is>
+          <t>84/199 (42%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="B236" s="20" t="inlineStr">
         <is>
           <t>Cobertura alvo (com INCLUIRs)</t>
         </is>
       </c>
-      <c r="C189" s="13" t="inlineStr">
-        <is>
-          <t>110/159 (69%)</t>
+      <c r="C236" s="13" t="inlineStr">
+        <is>
+          <t>142/199 (71%)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <mergeCells count="19">
+  <mergeCells count="26">
     <mergeCell ref="A153:L153"/>
+    <mergeCell ref="A217:L217"/>
+    <mergeCell ref="A208:L208"/>
     <mergeCell ref="A120:L120"/>
+    <mergeCell ref="A192:L192"/>
     <mergeCell ref="A105:L105"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A179:L179"/>
     <mergeCell ref="A42:L42"/>
     <mergeCell ref="A129:L129"/>
+    <mergeCell ref="A185:L185"/>
     <mergeCell ref="A141:L141"/>
     <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A180:L180"/>
     <mergeCell ref="A100:L100"/>
     <mergeCell ref="A147:L147"/>
     <mergeCell ref="A52:L52"/>
     <mergeCell ref="A170:L170"/>
     <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A202:L202"/>
     <mergeCell ref="A82:L82"/>
     <mergeCell ref="A166:L166"/>
     <mergeCell ref="A94:L94"/>
+    <mergeCell ref="A197:L197"/>
     <mergeCell ref="A70:L70"/>
     <mergeCell ref="A162:L162"/>
+    <mergeCell ref="A227:L227"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>